<commit_message>
Added median housing and income
</commit_message>
<xml_diff>
--- a/data/DataCollectionRedlining.xlsx
+++ b/data/DataCollectionRedlining.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29819"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wpi0-my.sharepoint.com/personal/ensalcedomarx_wpi_edu/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/54a1c0f8b736c45c/Documents/GitHub/final-theTeam/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{EA30B33D-7E91-7D45-B544-82A25159A8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34DD6B38-F0D6-4E52-A44A-586BDA427140}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{EA30B33D-7E91-7D45-B544-82A25159A8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBF3F42F-1422-43EC-909A-6FB440ED5DEB}"/>
   <bookViews>
-    <workbookView xWindow="5860" yWindow="580" windowWidth="27240" windowHeight="15360" xr2:uid="{AF438914-A1E0-4346-A623-7F68C664ED1A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{AF438914-A1E0-4346-A623-7F68C664ED1A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Zip Code</t>
   </si>
@@ -46,12 +46,6 @@
   <si>
     <t>Median Housing Price</t>
   </si>
-  <si>
-    <t>Unemployment Rate</t>
-  </si>
-  <si>
-    <t>Race and Ethnicity</t>
-  </si>
 </sst>
 </file>
 
@@ -60,7 +54,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="00000"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -190,7 +184,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!B1</c:f>
+              <c:f>Sheet1!$B$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -295,7 +289,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!C1</c:f>
+              <c:f>Sheet1!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1237,16 +1231,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>220980</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>89535</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>32385</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1591,16 +1585,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D670532-5452-904F-A3AA-C043C5D44646}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="23.1" customHeight="1">
+    <row r="1" spans="1:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1610,14 +1604,8 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" s="1" customFormat="1">
+    <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1602</v>
       </c>
@@ -1628,7 +1616,7 @@
         <v>438773</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="1" customFormat="1">
+    <row r="3" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1603</v>
       </c>
@@ -1639,7 +1627,7 @@
         <v>385207</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="1" customFormat="1">
+    <row r="4" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1604</v>
       </c>
@@ -1650,7 +1638,7 @@
         <v>409938</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1">
+    <row r="5" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>1605</v>
       </c>
@@ -1661,7 +1649,7 @@
         <v>431405</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="1" customFormat="1">
+    <row r="6" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>1606</v>
       </c>
@@ -1672,7 +1660,7 @@
         <v>428492</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="1" customFormat="1">
+    <row r="7" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>1607</v>
       </c>
@@ -1683,7 +1671,7 @@
         <v>377426</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="1" customFormat="1">
+    <row r="8" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>1608</v>
       </c>
@@ -1694,7 +1682,7 @@
         <v>187563</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="1" customFormat="1">
+    <row r="9" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>1609</v>
       </c>
@@ -1705,7 +1693,7 @@
         <v>529815</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="1" customFormat="1">
+    <row r="10" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>1610</v>
       </c>

</xml_diff>